<commit_message>
Add workbook config validation
</commit_message>
<xml_diff>
--- a/outputs/2026-06-27-tinh-split-stage3-enriched/TINH_MVP_engine_data_v0_7_source_clean.xlsx
+++ b/outputs/2026-06-27-tinh-split-stage3-enriched/TINH_MVP_engine_data_v0_7_source_clean.xlsx
@@ -876,7 +876,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -907,129 +907,139 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>meter.wellbeing.start</v>
+        <v>meter.openness.start</v>
       </c>
       <c r="B4" t="str">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="C4" t="str">
-        <v>S3 Tinh thần start</v>
+        <v>S2 openness start</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>meter.relationship.start</v>
+        <v>meter.wellbeing.start</v>
       </c>
       <c r="B5" t="str">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C5" t="str">
-        <v>S3 Tình thân start</v>
+        <v>S3 Tinh thần start</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>meter.clamp</v>
+        <v>meter.relationship.start</v>
       </c>
       <c r="B6" t="str">
-        <v>[0,100]</v>
+        <v>70</v>
       </c>
       <c r="C6" t="str">
-        <v>clamp every meter/openness</v>
+        <v>S3 Tình thân start</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>s1.customerCount</v>
+        <v>meter.clamp</v>
       </c>
       <c r="B7" t="str">
-        <v>2</v>
+        <v>[0,100]</v>
       </c>
       <c r="C7" t="str">
-        <v>MVP keeps C1 scam victim and C2 genuine customer</v>
+        <v>clamp every meter/openness</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>s1.requiredCatches</v>
+        <v>s1.customerCount</v>
       </c>
       <c r="B8" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="str">
-        <v>catch &gt;=1 victim to pass</v>
+        <v>MVP keeps C1 scam victim and C2 genuine customer</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>s1.genuineCount</v>
+        <v>s1.requiredCatches</v>
       </c>
       <c r="B9" t="str">
         <v>1</v>
       </c>
       <c r="C9" t="str">
-        <v>C2 only</v>
+        <v>catch &gt;=1 victim to pass</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>s1.passScore</v>
+        <v>s1.genuineCount</v>
       </c>
       <c r="B10" t="str">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C10" t="str">
-        <v>reachable in the two-customer MVP; max clean score is 16</v>
+        <v>C2 only</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>s1.repStart</v>
+        <v>s1.passScore</v>
       </c>
       <c r="B11" t="str">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="C11" t="str">
-        <v>Uy tín start</v>
+        <v>reachable in the two-customer MVP; max clean score is 16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>s2.enabledCases</v>
+        <v>s1.repStart</v>
       </c>
       <c r="B12" t="str">
-        <v>S2A</v>
+        <v>70</v>
       </c>
       <c r="C12" t="str">
-        <v>MVP keeps Bà Hạnh only</v>
+        <v>Uy tín start</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>flow</v>
+        <v>s2.enabledCases</v>
       </c>
       <c r="B13" t="str">
-        <v>s0→S1(C1,C2)→cs1→S2A→cs2→S3→ENDING</v>
+        <v>S2A</v>
       </c>
       <c r="C13" t="str">
-        <v>trimmed MVP order</v>
+        <v>MVP keeps Bà Hạnh only</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>flow</v>
+      </c>
+      <c r="B14" t="str">
+        <v>s0→S1(C1,C2)→cs1→S2A→cs2→S3→ENDING</v>
+      </c>
+      <c r="C14" t="str">
+        <v>trimmed MVP order</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>flow.firstBeat</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <v>s0_00</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C15" t="str">
         <v>boot into avatar select</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>